<commit_message>
Update tool and Supplementary File.
</commit_message>
<xml_diff>
--- a/SupplementaryFile.xlsx
+++ b/SupplementaryFile.xlsx
@@ -1,26 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thyang/SyncCloud/Works/Research/3_CRM/2022_CRM-gene_target/Supplementary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9544FB12-D1AF-C24A-BC96-4315E32A1BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45384202-DECD-6047-9AD7-278CE55B776C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4140" yWindow="600" windowWidth="28240" windowHeight="16460" activeTab="4" xr2:uid="{8995E919-6CB4-D04D-887A-1157242BEA27}"/>
+    <workbookView xWindow="5360" yWindow="600" windowWidth="28240" windowHeight="16460" activeTab="4" xr2:uid="{8995E919-6CB4-D04D-887A-1157242BEA27}"/>
   </bookViews>
   <sheets>
     <sheet name="TableS1" sheetId="2" r:id="rId1"/>
     <sheet name="TableS2" sheetId="3" r:id="rId2"/>
     <sheet name="Tables S3" sheetId="4" r:id="rId3"/>
     <sheet name="TableS4" sheetId="1" r:id="rId4"/>
-    <sheet name="Fig S1" sheetId="7" r:id="rId5"/>
-    <sheet name="Fig S2" sheetId="8" r:id="rId6"/>
-    <sheet name="Fig S3" sheetId="5" r:id="rId7"/>
-    <sheet name="Table S5" sheetId="6" r:id="rId8"/>
+    <sheet name="Fig S1" sheetId="9" r:id="rId5"/>
+    <sheet name="Fig S2" sheetId="7" r:id="rId6"/>
+    <sheet name="Fig S3" sheetId="8" r:id="rId7"/>
+    <sheet name="Fig S4" sheetId="5" r:id="rId8"/>
+    <sheet name="Fig S5" sheetId="11" r:id="rId9"/>
+    <sheet name="Table S5" sheetId="6" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="180">
   <si>
     <t>Training-validation Set</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -571,10 +573,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Fig S3: functional anlaysis of the genes regulated by different CRM regulatory mechanisms.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>a) Functional enrichment analysis for genes regulated by CRM-ncRNA transcription</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -587,15 +585,68 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Fig S2: comparison of CRM-TI with the average aggregation results of the two blocks in CRM-TI</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>(b) comparison of the random-initialized CRM-TI Block 2 model and the fine-tuned CRM-TI Block2 model</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">Fig S1:  (a) comparison of pre-training, fine-tuning results of CRM-TI Block 2 </t>
+    <t xml:space="preserve">Fig S1:  (a) length distribution of all CRMs with known target genes. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(c) The genomic distance between the non-overlapping CRM-target gene pairs.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> (b) The length distribution of the CRMs involving in the overlapping CRM-target gene pairs </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fig S4: functional anlaysis of the genes regulated by different CRM regulatory mechanisms.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fig S3: comparison of CRM-TI with the average aggregation results of the two blocks in CRM-TI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Fig S2:  (a) comparison of pre-training, fine-tuning results of CRM-TI Block 2 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fig S5: screenshots of the CRM-TI prediction results of the case study</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">chr3L_8711128_8120910 is the enhancer CRM while FBgn0001168 is the </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>hairy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> gene</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>d) The distribution of counts of known TFBSs within CRMs from all CRMs with known target genes.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>e) The distribution of counts of known TFBSs within CRMs from the non-overlapping CRM-target gene pairs</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -603,7 +654,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -620,6 +671,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -1082,6 +1140,231 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>15150</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="圖片 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D1C40450-21E5-EE13-58AA-16AC818A434F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="838200" y="6350000"/>
+          <a:ext cx="6606450" cy="3517900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>812800</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>112170</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="圖片 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EAA4EC1-8875-5ED0-9CB7-2B26832B4D14}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="838200" y="4254500"/>
+          <a:ext cx="6578600" cy="3503070"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>50799</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>131632</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="圖片 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BCC54BA4-F83D-122C-43E1-19C26E100234}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="838200" y="444499"/>
+          <a:ext cx="6591300" cy="3509833"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>15150</xdr:colOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="圖片 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E0E212F-BF1B-10C4-7716-B6F08C354A27}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="838200" y="12128500"/>
+          <a:ext cx="6606450" cy="3517900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>15150</xdr:colOff>
+      <xdr:row>104</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="圖片 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13C88CF5-0D79-138D-E5F2-A8E0D6292B20}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="838200" y="16116300"/>
+          <a:ext cx="6606450" cy="3517900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1218,7 +1501,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1267,7 +1550,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1393,6 +1676,55 @@
         <a:xfrm>
           <a:off x="1168400" y="6756400"/>
           <a:ext cx="4660900" cy="2997200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>355600</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>142790</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="圖片 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71E635AC-7438-20BF-74DB-21B18ECB46B9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="838200" y="546100"/>
+          <a:ext cx="7772400" cy="3038390"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1780,6 +2112,76 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF17D583-615F-7249-819A-C9FC179D3DAB}">
+  <dimension ref="B3:B14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="18.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:2" ht="16">
+      <c r="B3" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" ht="16" thickBot="1"/>
+    <row r="5" spans="2:2" ht="17" thickBot="1">
+      <c r="B5" s="18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" ht="16">
+      <c r="B6" s="19" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" ht="16">
+      <c r="B7" s="20" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" ht="16">
+      <c r="B8" s="20" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" ht="16">
+      <c r="B9" s="20" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" ht="16">
+      <c r="B10" s="20" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2" ht="16">
+      <c r="B11" s="20" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2" ht="16">
+      <c r="B12" s="20" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2" ht="16">
+      <c r="B13" s="20" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2" ht="17" thickBot="1">
+      <c r="B14" s="21" t="s">
+        <v>165</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{913D515B-8809-264A-B787-7E47DEF911DF}">
   <dimension ref="B3:C82"/>
@@ -2603,18 +3005,36 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F12322A1-B5D6-9547-B0AA-B4B75D3FF29E}">
-  <dimension ref="B2:B26"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D0A6EC3-9CD0-FF44-BF2B-4E9DF41F6172}">
+  <dimension ref="B2:B86"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="2:2" ht="16">
       <c r="B2" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" ht="16">
+      <c r="B23" s="1" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="26" spans="2:2" ht="16">
-      <c r="B26" s="1" t="s">
+    <row r="44" spans="2:2" ht="16">
+      <c r="B44" s="1" t="s">
         <v>171</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" ht="16">
+      <c r="B65" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" ht="16">
+      <c r="B66" s="1"/>
+    </row>
+    <row r="86" spans="2:2" ht="16">
+      <c r="B86" s="1" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -2625,13 +3045,18 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56F85087-E5D4-A54E-BED1-32BE084D7EC1}">
-  <dimension ref="B2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F12322A1-B5D6-9547-B0AA-B4B75D3FF29E}">
+  <dimension ref="B2:B26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="2:2" ht="16">
       <c r="B2" s="1" t="s">
-        <v>170</v>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" ht="16">
+      <c r="B26" s="1" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2642,6 +3067,23 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56F85087-E5D4-A54E-BED1-32BE084D7EC1}">
+  <dimension ref="B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2" spans="2:2" ht="16">
+      <c r="B2" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05B5B26-C09D-FB44-B90D-2CCECAD5E41F}">
   <dimension ref="B2:H34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
@@ -2651,17 +3093,17 @@
   <sheetData>
     <row r="2" spans="2:2" ht="16">
       <c r="B2" s="1" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="2:2" ht="16">
       <c r="B4" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="16">
       <c r="B17" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H17" s="1"/>
     </row>
@@ -2677,72 +3119,24 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF17D583-615F-7249-819A-C9FC179D3DAB}">
-  <dimension ref="B3:B14"/>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D635199-5F18-7742-8BAA-44DD6A823084}">
+  <dimension ref="B2:B20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="2" max="2" width="18.5" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="3" spans="2:2" ht="16">
-      <c r="B3" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="4" spans="2:2" ht="16" thickBot="1"/>
-    <row r="5" spans="2:2" ht="17" thickBot="1">
-      <c r="B5" s="18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="2:2" ht="16">
-      <c r="B6" s="19" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="7" spans="2:2" ht="16">
-      <c r="B7" s="20" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="8" spans="2:2" ht="16">
-      <c r="B8" s="20" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="9" spans="2:2" ht="16">
-      <c r="B9" s="20" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="10" spans="2:2" ht="16">
-      <c r="B10" s="20" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="11" spans="2:2" ht="16">
-      <c r="B11" s="20" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="12" spans="2:2" ht="16">
-      <c r="B12" s="20" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="13" spans="2:2" ht="16">
-      <c r="B13" s="20" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="14" spans="2:2" ht="17" thickBot="1">
-      <c r="B14" s="21" t="s">
-        <v>165</v>
+    <row r="2" spans="2:2" ht="16">
+      <c r="B2" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" ht="16">
+      <c r="B20" s="1" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>